<commit_message>
refactor(skills): 移除 dwm-data-inventory，清理步骤编号与 Kimball 标注
- 删除 dwm-data-inventory skill，输入改为直接读取 metadata_parse/ods_generator
- 新增 read_xlsx.py 共享工具
- write_bus_matrix.py 适配 xlsx 输入，调整列顺序为：主题域/业务过程/业务过程代码/粒度声明/事实表名称/事实表类型
- 清理所有带圈数字（②③⑤）和 Kimball Step 标注，改用 skill 名称引用
- 删除 dwm-matrix 步骤映射表，触发词下放到各 skill 自身 description
</commit_message>
<xml_diff>
--- a/output/dwm-bus-matrix/dwm_bus_matrix.xlsx
+++ b/output/dwm-bus-matrix/dwm_bus_matrix.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,16 +33,6 @@
     <font>
       <color rgb="00BDBDBD"/>
       <sz val="12"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="002E7D32"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00888888"/>
-      <sz val="9"/>
     </font>
   </fonts>
   <fills count="3">
@@ -77,7 +67,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -89,10 +79,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -458,18 +444,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="36" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -495,25 +482,30 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>事实表名称</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>事实表类型</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>优惠券维度</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>门店维度</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>商品维度</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>用户维度</t>
         </is>
@@ -542,25 +534,30 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
+          <t>dwd_inv_inventory_snapshot_df</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
           <t>periodic_snapshot</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -589,14 +586,14 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
+          <t>dwd_mkt_coupon_usage_df</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
           <t>factless</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
           <t>-</t>
@@ -607,9 +604,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -636,25 +638,30 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
+          <t>dwd_trd_order_detail_df</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
           <t>transaction</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -683,14 +690,14 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
+          <t>dwd_trd_payment_df</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
           <t>transaction</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
           <t>-</t>
@@ -701,9 +708,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -730,17 +742,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
+          <t>dwd_trd_place_order_df</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
           <t>transaction</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -748,9 +760,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -777,69 +794,32 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
+          <t>dwd_trd_refund_df</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
           <t>transaction</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>version</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>v1.0</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>published</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>updated_by</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>dwm-bus-matrix-skill</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>updated_at</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-10 21:43:12</t>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>